<commit_message>
Created set of cattle feed constraints that work with default rations
</commit_message>
<xml_diff>
--- a/data/scenarios/fix_default_feeddist.xlsx
+++ b/data/scenarios/fix_default_feeddist.xlsx
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="CattleHerd" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="162913" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="31">
   <si>
     <t>f_breed</t>
   </si>
@@ -47,18 +47,12 @@
     <t>drop</t>
   </si>
   <si>
-    <t>ley silage, 1st cut</t>
-  </si>
-  <si>
     <t>min_share_in_ration</t>
   </si>
   <si>
     <t>new</t>
   </si>
   <si>
-    <t>ley silage, regrowth</t>
-  </si>
-  <si>
     <t>max_DMI</t>
   </si>
   <si>
@@ -84,13 +78,55 @@
   </si>
   <si>
     <t>Drop fixed ley silage from rations</t>
+  </si>
+  <si>
+    <t>maize</t>
+  </si>
+  <si>
+    <t>If feed rations for cattle are completely fixed the solver finds the problem</t>
+  </si>
+  <si>
+    <t>infeasible. Likely due to some rounding errors. However if one feed is "set free"</t>
+  </si>
+  <si>
+    <t>it works.</t>
+  </si>
+  <si>
+    <t>Works with default rations</t>
+  </si>
+  <si>
+    <t>calves, suckling</t>
+  </si>
+  <si>
+    <t>Increased as default feed ration has &gt;50g/kg DM fat</t>
+  </si>
+  <si>
+    <t>dairy</t>
+  </si>
+  <si>
+    <t>cows</t>
+  </si>
+  <si>
+    <t>abs</t>
+  </si>
+  <si>
+    <t>Default factor (7.6) is much higher than default rations, especially organic dairy cows low (6.36). This is likely due to the 1:1 substitution of rapseed meal --&gt; rapseed cake in organic rations</t>
+  </si>
+  <si>
+    <t>Works with default rations after adjustments below</t>
+  </si>
+  <si>
+    <t>Organic dairy cows exceed 300 in default ration</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -120,6 +156,42 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="4"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -142,13 +214,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -342,14 +421,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="21" customWidth="1"/>
     <col min="3" max="4" width="21" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -366,13 +445,13 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G1" s="3"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="3"/>
@@ -381,9 +460,9 @@
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C3" s="1" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>5</v>
@@ -394,132 +473,222 @@
       <c r="F3">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="C4" s="1" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F4" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C5" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="H5" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="H7" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C8"/>
+      <c r="D8"/>
+      <c r="F8" s="10"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="1"/>
+      <c r="H9" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="10">
+        <v>6.3</v>
+      </c>
+      <c r="G10" s="10">
+        <v>7.6</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="B11" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11"/>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="10">
+        <v>6.1</v>
+      </c>
+      <c r="G11" s="10">
         <v>7</v>
       </c>
-      <c r="D5" s="1" t="s">
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C12"/>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F12" s="10">
+        <v>6.4</v>
+      </c>
+      <c r="G12" s="10">
+        <v>6.5</v>
+      </c>
+      <c r="H12" s="7"/>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C13"/>
+      <c r="D13"/>
+      <c r="F13" s="10"/>
+      <c r="H13" s="7"/>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="12"/>
+      <c r="T14" s="10"/>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="12"/>
+      <c r="J15" s="11"/>
+      <c r="T15" s="10"/>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D16" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" s="1"/>
+      <c r="J16" s="11"/>
+      <c r="T16" s="10"/>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="D17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F17" s="1"/>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="1">
+        <v>350</v>
+      </c>
+      <c r="G18">
+        <v>300</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="E19" s="4"/>
+      <c r="F19" s="1"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="D20" t="s">
+        <v>16</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F20" s="1"/>
+      <c r="H20" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B21" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" t="s">
+        <v>16</v>
+      </c>
+      <c r="E21" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F8" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F9" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D10" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F10" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F11" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D12" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F12" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D13" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F13" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D14" t="s">
-        <v>18</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="F14" s="1">
-        <v>1</v>
+      <c r="F21" s="1">
+        <v>100</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>